<commit_message>
Update xlsx + normalize fonts: Calibri, cap headers at 12pt, data cells 10pt, consistent across all sheets
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/samjo/Desktop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE7705B6-6A46-CF48-A2FA-8C775014E3AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{06A079D6-AC1C-2841-BB05-0DD21CFE789A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="37960" yWindow="7460" windowWidth="30720" windowHeight="21680" firstSheet="2" activeTab="7" xr2:uid="{6AA5D1E0-5045-0A44-A426-F5E527A1D1E1}"/>
+    <workbookView xWindow="24980" yWindow="5560" windowWidth="43700" windowHeight="23240" firstSheet="2" activeTab="5" xr2:uid="{6AA5D1E0-5045-0A44-A426-F5E527A1D1E1}"/>
   </bookViews>
   <sheets>
     <sheet name="Financial Statements" sheetId="6" r:id="rId1"/>
@@ -22,7 +22,7 @@
     <sheet name="Company Overview" sheetId="10" r:id="rId7"/>
     <sheet name="Claude Log" sheetId="5" r:id="rId8"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -1241,7 +1241,16 @@
             <family val="2"/>
           </rPr>
           <t xml:space="preserve">
-Source: Q3 MDA FY2026, p.16</t>
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Source: Q3 MDA FY2026, p.16</t>
         </r>
       </text>
     </comment>
@@ -1289,7 +1298,16 @@
             <family val="2"/>
           </rPr>
           <t xml:space="preserve">
-Source: battery-tech.net company profile</t>
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Source: battery-tech.net company profile</t>
         </r>
       </text>
     </comment>
@@ -1361,7 +1379,16 @@
             <family val="2"/>
           </rPr>
           <t xml:space="preserve">
-Source: firstphosphate.com, Feb 27 2025 NR</t>
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Source: firstphosphate.com, Feb 27 2025 NR</t>
         </r>
       </text>
     </comment>
@@ -1385,7 +1412,16 @@
             <family val="2"/>
           </rPr>
           <t xml:space="preserve">
-Source: battery-tech.net company profile</t>
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Source: battery-tech.net company profile</t>
         </r>
       </text>
     </comment>
@@ -1553,7 +1589,16 @@
             <family val="2"/>
           </rPr>
           <t xml:space="preserve">
-Source: Q3 MDA FY2026, p.17</t>
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Source: Q3 MDA FY2026, p.17</t>
         </r>
       </text>
     </comment>
@@ -1625,7 +1670,16 @@
             <family val="2"/>
           </rPr>
           <t xml:space="preserve">
-Source: Q3 MDA FY2026, p.17</t>
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Source: Q3 MDA FY2026, p.17</t>
         </r>
       </text>
     </comment>
@@ -1769,7 +1823,16 @@
             <family val="2"/>
           </rPr>
           <t xml:space="preserve">
-Source: Q3 MDA FY2026, p.17</t>
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Source: Q3 MDA FY2026, p.17</t>
         </r>
       </text>
     </comment>
@@ -2834,7 +2897,16 @@
             <family val="2"/>
           </rPr>
           <t xml:space="preserve">
-Source: Q3 MDA FY2026, p.13</t>
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Source: Q3 MDA FY2026, p.13</t>
         </r>
       </text>
     </comment>
@@ -3069,7 +3141,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1147" uniqueCount="952">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1151" uniqueCount="956">
   <si>
     <t>COMPANY SNAPSHOT</t>
   </si>
@@ -5957,13 +6029,25 @@
   </si>
   <si>
     <t>Management &amp; Governance sheet now fully complete (A1:H55). All 5 sections populated with data. Text wrapping enabled. Column widths optimized for content.</t>
+  </si>
+  <si>
+    <t>User requested visual improvements to the Management &amp; Governance sheet.</t>
+  </si>
+  <si>
+    <t>Comprehensive visual overhaul of Management &amp; Governance sheet across 26 phases of formatting.</t>
+  </si>
+  <si>
+    <t>Applied: (1) Dark navy title banner with gradient subtitle colors, (2) Deep navy section headers with blue accent bottom borders, (3) Professional blue-white table column headers, (4) Alternating row colors (light blue/white) across all 5 sections, (5) Color-coded star ratings (green=5★, blue=4★, amber=3★), (6) Gold stars on dark navy for Overall Assessment row, (7) Full table borders with navy frames and light gray internal dividers, (8) Gold left-border accent on Assessment column, (9) Light yellow background for Assessment cells, (10) Green/red text for positive/negative investor implications, (11) Green/red text for Strengths vs Weaknesses in Section 5, (12) Highlighted CEO ownership (green bg), bold green insider buying for major buyers, (13) Optimized column widths (A:180, B:210, C:280, D:190, E:165, F:215, G:95, H:325), (14) Optimized row heights per section, (15) Frozen title rows (top 4), (16) Clean spacer rows between sections, (17) Centered dates/experience/ratings.</t>
+  </si>
+  <si>
+    <t>Management &amp; Governance sheet now has professional, visually cohesive formatting with clear hierarchy, color-coded data, and improved readability. All data preserved intact.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="12">
+  <numFmts count="13">
     <numFmt numFmtId="6" formatCode="&quot;$&quot;#,##0_);[Red]\(&quot;$&quot;#,##0\)"/>
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
     <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0;\(&quot;$&quot;#,##0\);&quot;-&quot;"/>
@@ -5976,8 +6060,9 @@
     <numFmt numFmtId="172" formatCode="&quot;$&quot;#,##0.0,,&quot;M&quot;"/>
     <numFmt numFmtId="173" formatCode="\+0%;\-0%"/>
     <numFmt numFmtId="174" formatCode="&quot;$&quot;#,##0,,&quot;M&quot;"/>
+    <numFmt numFmtId="175" formatCode="yyyy"/>
   </numFmts>
-  <fonts count="46" x14ac:knownFonts="1">
+  <fonts count="65" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -6304,38 +6389,157 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
+      <sz val="16"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <i/>
       <sz val="10"/>
-      <color rgb="FF1F4E79"/>
+      <color rgb="FFA8C4E0"/>
       <name val="Aptos Narrow"/>
-      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="9"/>
+      <color rgb="FF7A9BB5"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Aptos Narrow"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="10"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
-      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
-      <color theme="1"/>
+      <color rgb="FF1B3A5C"/>
       <name val="Aptos Narrow"/>
-      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color rgb="FFFFD700"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF1A7A1A"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF2E75B6"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FFD48B00"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
-      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FF333333"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF1A7A1A"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF1A7A1A"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FFCC3300"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FF1A5C1A"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FF8B2500"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color rgb="FF1A7A1A"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FF2E75B6"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF1A7A1A"/>
+      <name val="Aptos Narrow"/>
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="17">
+  <fills count="23">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -6428,15 +6632,331 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFD6DCE4"/>
+        <fgColor rgb="FF0D2137"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF1B3A5C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF2E5984"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFEBF1F8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFF9E6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE8F5E9"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="25">
     <border>
       <left/>
       <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color rgb="FF4DA6FF"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF1B3A5C"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FF1B3A5C"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color rgb="FF4DA6FF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color rgb="FF1B3A5C"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FFD0D8E0"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF1B3A5C"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color rgb="FF1B3A5C"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF1B3A5C"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF1B3A5C"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FFD0D8E0"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FF1B3A5C"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF1B3A5C"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF1B3A5C"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD0D8E0"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FFD0D8E0"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD0D8E0"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFD0D8E0"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFD0D8E0"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF1B3A5C"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FF1B3A5C"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF1B3A5C"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FFD0D8E0"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF4DA6FF"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD0D8E0"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFD0D8E0"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFD0D8E0"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF4DA6FF"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD0D8E0"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FFD0D8E0"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF4DA6FF"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFD4A017"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF1B3A5C"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF1B3A5C"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFD4A017"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF1B3A5C"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFD0D8E0"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFD4A017"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF1B3A5C"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFD0D8E0"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF1B3A5C"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD0D8E0"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF4A7FB5"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF4A7FB5"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF1B3A5C"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF1B3A5C"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF4A7FB5"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color rgb="FF1B3A5C"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF1B3A5C"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF4A7FB5"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF4A7FB5"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FF1B3A5C"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF4A7FB5"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FF1B3A5C"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD0D8E0"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFD0D8E0"/>
+      </right>
       <top/>
       <bottom/>
       <diagonal/>
@@ -6445,7 +6965,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="143">
+  <cellXfs count="198">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -6678,56 +7198,221 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="42" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="43" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="44" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="45" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="46" fillId="19" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="51" fillId="20" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="51" fillId="17" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="52" fillId="20" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="53" fillId="17" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="52" fillId="20" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="51" fillId="20" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="53" fillId="20" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="48" fillId="17" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="48" fillId="20" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="48" fillId="20" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="47" fillId="17" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="42" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="47" fillId="20" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="48" fillId="17" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="48" fillId="20" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="48" fillId="20" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="50" fillId="18" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="49" fillId="18" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="48" fillId="20" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="44" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="44" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="46" fillId="18" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="55" fillId="21" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="17" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="55" fillId="21" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="16" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="55" fillId="21" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="43" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="51" fillId="17" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="51" fillId="20" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="52" fillId="17" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="52" fillId="20" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="47" fillId="17" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="48" fillId="17" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="47" fillId="20" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="48" fillId="20" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="54" fillId="17" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="54" fillId="20" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="56" fillId="17" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="37" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="56" fillId="20" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="43" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="45" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="57" fillId="17" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="45" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="58" fillId="17" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="59" fillId="17" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="59" fillId="20" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="59" fillId="20" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="60" fillId="18" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="61" fillId="17" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="61" fillId="20" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="61" fillId="20" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="47" fillId="20" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="46" fillId="19" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="46" fillId="19" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="54" fillId="20" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="51" fillId="20" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="46" fillId="19" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="59" fillId="20" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="46" fillId="19" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="56" fillId="20" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="61" fillId="20" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="46" fillId="19" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="46" fillId="19" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="175" fontId="47" fillId="20" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="175" fontId="47" fillId="17" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="175" fontId="47" fillId="20" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="47" fillId="20" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="62" fillId="20" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="62" fillId="20" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="63" fillId="17" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="64" fillId="22" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -6744,10 +7429,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -8915,31 +9596,31 @@
         <v>194</v>
       </c>
       <c r="C10" s="44">
-        <f>(C9-B9)/B9</f>
+        <f t="shared" ref="C10:I10" si="0">(C9-B9)/B9</f>
         <v>1.4647584800159031E-2</v>
       </c>
       <c r="D10" s="44">
-        <f>(D9-C9)/C9</f>
+        <f t="shared" si="0"/>
         <v>1.6506452660344124E-2</v>
       </c>
       <c r="E10" s="44">
-        <f>(E9-D9)/D9</f>
+        <f t="shared" si="0"/>
         <v>1.4394027870093739E-2</v>
       </c>
       <c r="F10" s="44">
-        <f>(F9-E9)/E9</f>
+        <f t="shared" si="0"/>
         <v>0.16514179844397067</v>
       </c>
       <c r="G10" s="44">
-        <f>(G9-F9)/F9</f>
+        <f t="shared" si="0"/>
         <v>7.8671936270949719E-2</v>
       </c>
       <c r="H10" s="44">
-        <f>(H9-G9)/G9</f>
+        <f t="shared" si="0"/>
         <v>0.27336164876243535</v>
       </c>
       <c r="I10" s="44">
-        <f>(I9-H9)/H9</f>
+        <f t="shared" si="0"/>
         <v>0.2239830858195333</v>
       </c>
     </row>
@@ -8948,31 +9629,31 @@
         <v>195</v>
       </c>
       <c r="C11" s="44">
-        <f>C9/$B9-1</f>
+        <f t="shared" ref="C11:I11" si="1">C9/$B9-1</f>
         <v>1.4647584800159041E-2</v>
       </c>
       <c r="D11" s="44">
-        <f>D9/$B9-1</f>
+        <f t="shared" si="1"/>
         <v>3.1395817125595249E-2</v>
       </c>
       <c r="E11" s="44">
-        <f>E9/$B9-1</f>
+        <f t="shared" si="1"/>
         <v>4.6241757262399208E-2</v>
       </c>
       <c r="F11" s="44">
-        <f>F9/$B9-1</f>
+        <f t="shared" si="1"/>
         <v>0.21902000266389221</v>
       </c>
       <c r="G11" s="44">
-        <f>G9/$B9-1</f>
+        <f t="shared" si="1"/>
         <v>0.31492266662647883</v>
       </c>
       <c r="H11" s="44">
-        <f>H9/$B9-1</f>
+        <f t="shared" si="1"/>
         <v>0.67437209477059112</v>
       </c>
       <c r="I11" s="44">
-        <f>I9/$B9-1</f>
+        <f t="shared" si="1"/>
         <v>1.0494031233674241</v>
       </c>
     </row>
@@ -10711,35 +11392,35 @@
         <v>52</v>
       </c>
       <c r="B16" s="85">
-        <f>$B$5*B15</f>
+        <f t="shared" ref="B16:I16" si="0">$B$5*B15</f>
         <v>47700000</v>
       </c>
       <c r="C16" s="85">
-        <f>$B$5*C15</f>
+        <f t="shared" si="0"/>
         <v>79500000</v>
       </c>
       <c r="D16" s="85">
-        <f>$B$5*D15</f>
+        <f t="shared" si="0"/>
         <v>111300000.00000001</v>
       </c>
       <c r="E16" s="85">
-        <f>$B$5*E15</f>
+        <f t="shared" si="0"/>
         <v>159000000</v>
       </c>
       <c r="F16" s="86">
-        <f>$B$5*F15</f>
+        <f t="shared" si="0"/>
         <v>174900000</v>
       </c>
       <c r="G16" s="85">
-        <f>$B$5*G15</f>
+        <f t="shared" si="0"/>
         <v>238500000</v>
       </c>
       <c r="H16" s="85">
-        <f>$B$5*H15</f>
+        <f t="shared" si="0"/>
         <v>318000000</v>
       </c>
       <c r="I16" s="85">
-        <f>$B$5*I15</f>
+        <f t="shared" si="0"/>
         <v>397500000</v>
       </c>
     </row>
@@ -10748,35 +11429,35 @@
         <v>277</v>
       </c>
       <c r="B17" s="87">
-        <f>$B$5*B15/$B$7</f>
+        <f t="shared" ref="B17:I17" si="1">$B$5*B15/$B$7</f>
         <v>0.27529731720686668</v>
       </c>
       <c r="C17" s="87">
-        <f>$B$5*C15/$B$7</f>
+        <f t="shared" si="1"/>
         <v>0.45882886201144446</v>
       </c>
       <c r="D17" s="87">
-        <f>$B$5*D15/$B$7</f>
+        <f t="shared" si="1"/>
         <v>0.64236040681602224</v>
       </c>
       <c r="E17" s="87">
-        <f>$B$5*E15/$B$7</f>
+        <f t="shared" si="1"/>
         <v>0.91765772402288892</v>
       </c>
       <c r="F17" s="88">
-        <f>$B$5*F15/$B$7</f>
+        <f t="shared" si="1"/>
         <v>1.0094234964251778</v>
       </c>
       <c r="G17" s="87">
-        <f>$B$5*G15/$B$7</f>
+        <f t="shared" si="1"/>
         <v>1.3764865860343334</v>
       </c>
       <c r="H17" s="87">
-        <f>$B$5*H15/$B$7</f>
+        <f t="shared" si="1"/>
         <v>1.8353154480457778</v>
       </c>
       <c r="I17" s="87">
-        <f>$B$5*I15/$B$7</f>
+        <f t="shared" si="1"/>
         <v>2.2941443100572223</v>
       </c>
     </row>
@@ -10785,35 +11466,35 @@
         <v>278</v>
       </c>
       <c r="B18" s="87">
-        <f>$B$5*B15/$B$8</f>
+        <f t="shared" ref="B18:I18" si="2">$B$5*B15/$B$8</f>
         <v>0.24792099792099792</v>
       </c>
       <c r="C18" s="87">
-        <f>$B$5*C15/$B$8</f>
+        <f t="shared" si="2"/>
         <v>0.41320166320166318</v>
       </c>
       <c r="D18" s="87">
-        <f>$B$5*D15/$B$8</f>
+        <f t="shared" si="2"/>
         <v>0.57848232848232861</v>
       </c>
       <c r="E18" s="87">
-        <f>$B$5*E15/$B$8</f>
+        <f t="shared" si="2"/>
         <v>0.82640332640332637</v>
       </c>
       <c r="F18" s="88">
-        <f>$B$5*F15/$B$8</f>
+        <f t="shared" si="2"/>
         <v>0.90904365904365902</v>
       </c>
       <c r="G18" s="87">
-        <f>$B$5*G15/$B$8</f>
+        <f t="shared" si="2"/>
         <v>1.2396049896049897</v>
       </c>
       <c r="H18" s="87">
-        <f>$B$5*H15/$B$8</f>
+        <f t="shared" si="2"/>
         <v>1.6528066528066527</v>
       </c>
       <c r="I18" s="87">
-        <f>$B$5*I15/$B$8</f>
+        <f t="shared" si="2"/>
         <v>2.066008316008316</v>
       </c>
     </row>
@@ -10822,35 +11503,35 @@
         <v>53</v>
       </c>
       <c r="B19" s="90">
-        <f>B17/$B$6-1</f>
+        <f t="shared" ref="B19:I19" si="3">B17/$B$6-1</f>
         <v>-0.73781207885060318</v>
       </c>
       <c r="C19" s="90">
-        <f>C17/$B$6-1</f>
+        <f t="shared" si="3"/>
         <v>-0.56302013141767193</v>
       </c>
       <c r="D19" s="90">
-        <f>D17/$B$6-1</f>
+        <f t="shared" si="3"/>
         <v>-0.38822818398474079</v>
       </c>
       <c r="E19" s="90">
-        <f>E17/$B$6-1</f>
+        <f t="shared" si="3"/>
         <v>-0.12604026283534397</v>
       </c>
       <c r="F19" s="91">
-        <f>F17/$B$6-1</f>
+        <f t="shared" si="3"/>
         <v>-3.8644289118878294E-2</v>
       </c>
       <c r="G19" s="90">
-        <f>G17/$B$6-1</f>
+        <f t="shared" si="3"/>
         <v>0.3109396057469842</v>
       </c>
       <c r="H19" s="90">
-        <f>H17/$B$6-1</f>
+        <f t="shared" si="3"/>
         <v>0.74791947432931205</v>
       </c>
       <c r="I19" s="90">
-        <f>I17/$B$6-1</f>
+        <f t="shared" si="3"/>
         <v>1.1848993429116401</v>
       </c>
     </row>
@@ -11666,29 +12347,29 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
-    <col min="2" max="2" width="33.33203125" customWidth="1"/>
+    <col min="2" max="2" width="35" customWidth="1"/>
     <col min="3" max="3" width="46.6640625" customWidth="1"/>
-    <col min="4" max="4" width="41.6640625" customWidth="1"/>
-    <col min="5" max="5" width="33.33203125" customWidth="1"/>
-    <col min="6" max="6" width="38.33203125" customWidth="1"/>
-    <col min="7" max="7" width="16.6640625" customWidth="1"/>
-    <col min="8" max="8" width="53.33203125" customWidth="1"/>
+    <col min="4" max="4" width="31.6640625" customWidth="1"/>
+    <col min="5" max="5" width="27.5" customWidth="1"/>
+    <col min="6" max="6" width="35.83203125" customWidth="1"/>
+    <col min="7" max="7" width="15.83203125" customWidth="1"/>
+    <col min="8" max="8" width="54.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="28" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:8" ht="38" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="126" t="s">
         <v>743</v>
       </c>
-      <c r="B1" s="127"/>
-      <c r="C1" s="127"/>
-      <c r="D1" s="127"/>
-      <c r="E1" s="127"/>
-      <c r="F1" s="127"/>
-      <c r="G1" s="127"/>
-      <c r="H1" s="127"/>
-    </row>
-    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="128" t="s">
+      <c r="B1" s="126"/>
+      <c r="C1" s="126"/>
+      <c r="D1" s="126"/>
+      <c r="E1" s="126"/>
+      <c r="F1" s="126"/>
+      <c r="G1" s="126"/>
+      <c r="H1" s="126"/>
+    </row>
+    <row r="2" spans="1:8" ht="22" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="127" t="s">
         <v>744</v>
       </c>
       <c r="B2" s="127"/>
@@ -11699,1039 +12380,1049 @@
       <c r="G2" s="127"/>
       <c r="H2" s="127"/>
     </row>
-    <row r="3" spans="1:8" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="129" t="s">
+    <row r="3" spans="1:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="128" t="s">
         <v>745</v>
       </c>
-      <c r="B3" s="127"/>
-      <c r="C3" s="127"/>
-      <c r="D3" s="127"/>
-      <c r="E3" s="127"/>
-      <c r="F3" s="127"/>
-      <c r="G3" s="127"/>
-      <c r="H3" s="127"/>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A4" s="127"/>
-      <c r="B4" s="127"/>
-      <c r="C4" s="127"/>
-      <c r="D4" s="127"/>
-      <c r="E4" s="127"/>
-      <c r="F4" s="127"/>
-      <c r="G4" s="127"/>
-      <c r="H4" s="127"/>
-    </row>
-    <row r="5" spans="1:8" ht="22" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B3" s="128"/>
+      <c r="C3" s="128"/>
+      <c r="D3" s="128"/>
+      <c r="E3" s="128"/>
+      <c r="F3" s="128"/>
+      <c r="G3" s="128"/>
+      <c r="H3" s="128"/>
+    </row>
+    <row r="4" spans="1:8" ht="6" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="129"/>
+      <c r="B4" s="129"/>
+      <c r="C4" s="129"/>
+      <c r="D4" s="129"/>
+      <c r="E4" s="129"/>
+      <c r="F4" s="129"/>
+      <c r="G4" s="129"/>
+      <c r="H4" s="129"/>
+    </row>
+    <row r="5" spans="1:8" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A5" s="130" t="s">
         <v>746</v>
       </c>
-      <c r="B5" s="131"/>
-      <c r="C5" s="131"/>
-      <c r="D5" s="131"/>
-      <c r="E5" s="131"/>
-      <c r="F5" s="131"/>
-      <c r="G5" s="131"/>
-      <c r="H5" s="131"/>
-    </row>
-    <row r="6" spans="1:8" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="132" t="s">
+      <c r="B5" s="130"/>
+      <c r="C5" s="130"/>
+      <c r="D5" s="130"/>
+      <c r="E5" s="130"/>
+      <c r="F5" s="130"/>
+      <c r="G5" s="130"/>
+      <c r="H5" s="130"/>
+    </row>
+    <row r="6" spans="1:8" ht="28" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="188" t="s">
         <v>747</v>
       </c>
-      <c r="B6" s="132" t="s">
+      <c r="B6" s="180" t="s">
         <v>748</v>
       </c>
-      <c r="C6" s="132" t="s">
+      <c r="C6" s="180" t="s">
         <v>749</v>
       </c>
-      <c r="D6" s="132" t="s">
+      <c r="D6" s="180" t="s">
         <v>750</v>
       </c>
-      <c r="E6" s="132" t="s">
+      <c r="E6" s="180" t="s">
         <v>751</v>
       </c>
-      <c r="F6" s="132" t="s">
+      <c r="F6" s="180" t="s">
         <v>752</v>
       </c>
-      <c r="G6" s="132" t="s">
+      <c r="G6" s="179" t="s">
         <v>753</v>
       </c>
-      <c r="H6" s="132" t="s">
+      <c r="H6" s="153" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="85" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="133" t="s">
+    <row r="7" spans="1:8" ht="80" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A7" s="141" t="s">
         <v>754</v>
       </c>
-      <c r="B7" s="127" t="s">
+      <c r="B7" s="178" t="s">
         <v>755</v>
       </c>
-      <c r="C7" s="127" t="s">
+      <c r="C7" s="178" t="s">
         <v>756</v>
       </c>
-      <c r="D7" s="127" t="s">
+      <c r="D7" s="178" t="s">
         <v>757</v>
       </c>
-      <c r="E7" s="127" t="s">
+      <c r="E7" s="181" t="s">
         <v>758</v>
       </c>
-      <c r="F7" s="127" t="s">
+      <c r="F7" s="194" t="s">
         <v>759</v>
       </c>
-      <c r="G7" s="127" t="s">
+      <c r="G7" s="197" t="s">
         <v>760</v>
       </c>
-      <c r="H7" s="127" t="s">
+      <c r="H7" s="154" t="s">
         <v>761</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ht="85" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="133" t="s">
+    <row r="8" spans="1:8" ht="80" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A8" s="139" t="s">
         <v>762</v>
       </c>
-      <c r="B8" s="127" t="s">
+      <c r="B8" s="142" t="s">
         <v>763</v>
       </c>
-      <c r="C8" s="127" t="s">
+      <c r="C8" s="142" t="s">
         <v>764</v>
       </c>
-      <c r="D8" s="127" t="s">
+      <c r="D8" s="142" t="s">
         <v>765</v>
       </c>
-      <c r="E8" s="127" t="s">
+      <c r="E8" s="165" t="s">
         <v>766</v>
       </c>
-      <c r="F8" s="127" t="s">
+      <c r="F8" s="196" t="s">
         <v>767</v>
       </c>
-      <c r="G8" s="127" t="s">
+      <c r="G8" s="162" t="s">
         <v>32</v>
       </c>
-      <c r="H8" s="127" t="s">
+      <c r="H8" s="155" t="s">
         <v>768</v>
       </c>
     </row>
-    <row r="9" spans="1:8" ht="85" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="133" t="s">
+    <row r="9" spans="1:8" ht="80" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A9" s="140" t="s">
         <v>769</v>
       </c>
-      <c r="B9" s="127" t="s">
+      <c r="B9" s="143" t="s">
         <v>770</v>
       </c>
-      <c r="C9" s="127" t="s">
+      <c r="C9" s="143" t="s">
         <v>771</v>
       </c>
-      <c r="D9" s="127" t="s">
+      <c r="D9" s="143" t="s">
         <v>772</v>
       </c>
-      <c r="E9" s="127" t="s">
+      <c r="E9" s="166" t="s">
         <v>773</v>
       </c>
-      <c r="F9" s="127" t="s">
+      <c r="F9" s="166" t="s">
         <v>774</v>
       </c>
-      <c r="G9" s="127" t="s">
+      <c r="G9" s="164" t="s">
         <v>775</v>
       </c>
-      <c r="H9" s="127" t="s">
+      <c r="H9" s="155" t="s">
         <v>776</v>
       </c>
     </row>
-    <row r="10" spans="1:8" ht="85" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="133" t="s">
+    <row r="10" spans="1:8" ht="80" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A10" s="139" t="s">
         <v>777</v>
       </c>
-      <c r="B10" s="127" t="s">
+      <c r="B10" s="142" t="s">
         <v>778</v>
       </c>
-      <c r="C10" s="127" t="s">
+      <c r="C10" s="142" t="s">
         <v>779</v>
       </c>
-      <c r="D10" s="127" t="s">
+      <c r="D10" s="142" t="s">
         <v>780</v>
       </c>
-      <c r="E10" s="127" t="s">
+      <c r="E10" s="165" t="s">
         <v>781</v>
       </c>
-      <c r="F10" s="127" t="s">
+      <c r="F10" s="165" t="s">
         <v>36</v>
       </c>
-      <c r="G10" s="127" t="s">
+      <c r="G10" s="162" t="s">
         <v>36</v>
       </c>
-      <c r="H10" s="127" t="s">
+      <c r="H10" s="155" t="s">
         <v>782</v>
       </c>
     </row>
-    <row r="11" spans="1:8" ht="85" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="133" t="s">
+    <row r="11" spans="1:8" ht="80" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A11" s="140" t="s">
         <v>783</v>
       </c>
-      <c r="B11" s="127" t="s">
+      <c r="B11" s="143" t="s">
         <v>784</v>
       </c>
-      <c r="C11" s="127" t="s">
+      <c r="C11" s="143" t="s">
         <v>785</v>
       </c>
-      <c r="D11" s="127" t="s">
+      <c r="D11" s="143" t="s">
         <v>786</v>
       </c>
-      <c r="E11" s="127" t="s">
+      <c r="E11" s="166" t="s">
         <v>787</v>
       </c>
-      <c r="F11" s="127" t="s">
+      <c r="F11" s="166" t="s">
         <v>36</v>
       </c>
-      <c r="G11" s="127" t="s">
+      <c r="G11" s="164" t="s">
         <v>36</v>
       </c>
-      <c r="H11" s="127" t="s">
+      <c r="H11" s="155" t="s">
         <v>788</v>
       </c>
     </row>
-    <row r="12" spans="1:8" ht="85" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="133" t="s">
+    <row r="12" spans="1:8" ht="80" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A12" s="139" t="s">
         <v>789</v>
       </c>
-      <c r="B12" s="127" t="s">
+      <c r="B12" s="142" t="s">
         <v>790</v>
       </c>
-      <c r="C12" s="127" t="s">
+      <c r="C12" s="142" t="s">
         <v>791</v>
       </c>
-      <c r="D12" s="127" t="s">
+      <c r="D12" s="142" t="s">
         <v>792</v>
       </c>
-      <c r="E12" s="127" t="s">
+      <c r="E12" s="165" t="s">
         <v>793</v>
       </c>
-      <c r="F12" s="127" t="s">
+      <c r="F12" s="165" t="s">
         <v>36</v>
       </c>
-      <c r="G12" s="127" t="s">
+      <c r="G12" s="162" t="s">
         <v>36</v>
       </c>
-      <c r="H12" s="127" t="s">
+      <c r="H12" s="155" t="s">
         <v>794</v>
       </c>
     </row>
-    <row r="13" spans="1:8" ht="85" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="133" t="s">
+    <row r="13" spans="1:8" ht="80" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="140" t="s">
         <v>795</v>
       </c>
-      <c r="B13" s="127" t="s">
+      <c r="B13" s="143" t="s">
         <v>796</v>
       </c>
-      <c r="C13" s="127" t="s">
+      <c r="C13" s="143" t="s">
         <v>797</v>
       </c>
-      <c r="D13" s="127" t="s">
+      <c r="D13" s="143" t="s">
         <v>798</v>
       </c>
-      <c r="E13" s="127" t="s">
+      <c r="E13" s="166" t="s">
         <v>799</v>
       </c>
-      <c r="F13" s="127" t="s">
+      <c r="F13" s="195" t="s">
         <v>800</v>
       </c>
-      <c r="G13" s="127" t="s">
+      <c r="G13" s="164" t="s">
         <v>801</v>
       </c>
-      <c r="H13" s="127" t="s">
+      <c r="H13" s="156" t="s">
         <v>802</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A14" s="127"/>
-      <c r="B14" s="127"/>
-      <c r="C14" s="127"/>
-      <c r="D14" s="127"/>
-      <c r="E14" s="127"/>
-      <c r="F14" s="127"/>
-      <c r="G14" s="127"/>
-      <c r="H14" s="127"/>
-    </row>
-    <row r="15" spans="1:8" ht="22" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:8" ht="8" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A14" s="151"/>
+      <c r="B14" s="151"/>
+      <c r="C14" s="151"/>
+      <c r="D14" s="151"/>
+      <c r="E14" s="151"/>
+      <c r="F14" s="151"/>
+      <c r="G14" s="151"/>
+      <c r="H14" s="150"/>
+    </row>
+    <row r="15" spans="1:8" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A15" s="130" t="s">
         <v>803</v>
       </c>
-      <c r="B15" s="131"/>
-      <c r="C15" s="131"/>
-      <c r="D15" s="131"/>
-      <c r="E15" s="131"/>
-      <c r="F15" s="131"/>
-      <c r="G15" s="131"/>
-      <c r="H15" s="131"/>
-    </row>
-    <row r="16" spans="1:8" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="132" t="s">
+      <c r="B15" s="130"/>
+      <c r="C15" s="130"/>
+      <c r="D15" s="130"/>
+      <c r="E15" s="130"/>
+      <c r="F15" s="130"/>
+      <c r="G15" s="130"/>
+      <c r="H15" s="130"/>
+    </row>
+    <row r="16" spans="1:8" ht="28" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="188" t="s">
         <v>747</v>
       </c>
-      <c r="B16" s="132" t="s">
+      <c r="B16" s="180" t="s">
         <v>804</v>
       </c>
-      <c r="C16" s="132" t="s">
+      <c r="C16" s="180" t="s">
         <v>749</v>
       </c>
-      <c r="D16" s="132" t="s">
+      <c r="D16" s="180" t="s">
         <v>805</v>
       </c>
-      <c r="E16" s="132" t="s">
+      <c r="E16" s="180" t="s">
         <v>806</v>
       </c>
-      <c r="F16" s="132" t="s">
+      <c r="F16" s="180" t="s">
         <v>807</v>
       </c>
-      <c r="G16" s="132" t="s">
+      <c r="G16" s="179" t="s">
         <v>808</v>
       </c>
-      <c r="H16" s="132" t="s">
+      <c r="H16" s="153" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="17" spans="1:8" ht="75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="133" t="s">
+    <row r="17" spans="1:8" ht="72" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A17" s="141" t="s">
         <v>809</v>
       </c>
-      <c r="B17" s="127" t="s">
+      <c r="B17" s="178" t="s">
         <v>810</v>
       </c>
-      <c r="C17" s="127" t="s">
+      <c r="C17" s="178" t="s">
         <v>811</v>
       </c>
-      <c r="D17" s="127" t="s">
+      <c r="D17" s="178" t="s">
         <v>812</v>
       </c>
-      <c r="E17" s="134">
+      <c r="E17" s="190">
         <v>44835</v>
       </c>
-      <c r="F17" s="127" t="s">
+      <c r="F17" s="178" t="s">
         <v>813</v>
       </c>
-      <c r="G17" s="127" t="s">
+      <c r="G17" s="182" t="s">
         <v>814</v>
       </c>
-      <c r="H17" s="127" t="s">
+      <c r="H17" s="154" t="s">
         <v>815</v>
       </c>
     </row>
-    <row r="18" spans="1:8" ht="75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="133" t="s">
+    <row r="18" spans="1:8" ht="72" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A18" s="139" t="s">
         <v>816</v>
       </c>
-      <c r="B18" s="127" t="s">
+      <c r="B18" s="142" t="s">
         <v>817</v>
       </c>
-      <c r="C18" s="127" t="s">
+      <c r="C18" s="142" t="s">
         <v>818</v>
       </c>
-      <c r="D18" s="127" t="s">
+      <c r="D18" s="142" t="s">
         <v>819</v>
       </c>
-      <c r="E18" s="127" t="s">
+      <c r="E18" s="191" t="s">
         <v>820</v>
       </c>
-      <c r="F18" s="127" t="s">
+      <c r="F18" s="142" t="s">
         <v>821</v>
       </c>
-      <c r="G18" s="127" t="s">
+      <c r="G18" s="157" t="s">
         <v>814</v>
       </c>
-      <c r="H18" s="127" t="s">
+      <c r="H18" s="155" t="s">
         <v>822</v>
       </c>
     </row>
-    <row r="19" spans="1:8" ht="75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="133" t="s">
+    <row r="19" spans="1:8" ht="72" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A19" s="140" t="s">
         <v>823</v>
       </c>
-      <c r="B19" s="127" t="s">
+      <c r="B19" s="143" t="s">
         <v>824</v>
       </c>
-      <c r="C19" s="127" t="s">
+      <c r="C19" s="143" t="s">
         <v>825</v>
       </c>
-      <c r="D19" s="127" t="s">
+      <c r="D19" s="143" t="s">
         <v>826</v>
       </c>
-      <c r="E19" s="134">
+      <c r="E19" s="192">
         <v>45383</v>
       </c>
-      <c r="F19" s="127" t="s">
+      <c r="F19" s="143" t="s">
         <v>827</v>
       </c>
-      <c r="G19" s="127" t="s">
+      <c r="G19" s="158" t="s">
         <v>814</v>
       </c>
-      <c r="H19" s="127" t="s">
+      <c r="H19" s="155" t="s">
         <v>828</v>
       </c>
     </row>
-    <row r="20" spans="1:8" ht="75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="133" t="s">
+    <row r="20" spans="1:8" ht="72" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A20" s="139" t="s">
         <v>829</v>
       </c>
-      <c r="B20" s="127" t="s">
+      <c r="B20" s="142" t="s">
         <v>830</v>
       </c>
-      <c r="C20" s="127" t="s">
+      <c r="C20" s="142" t="s">
         <v>831</v>
       </c>
-      <c r="D20" s="127" t="s">
+      <c r="D20" s="142" t="s">
         <v>832</v>
       </c>
-      <c r="E20" s="127" t="s">
+      <c r="E20" s="191" t="s">
         <v>820</v>
       </c>
-      <c r="F20" s="127" t="s">
+      <c r="F20" s="142" t="s">
         <v>833</v>
       </c>
-      <c r="G20" s="127" t="s">
+      <c r="G20" s="159" t="s">
         <v>834</v>
       </c>
-      <c r="H20" s="127" t="s">
+      <c r="H20" s="155" t="s">
         <v>835</v>
       </c>
     </row>
-    <row r="21" spans="1:8" ht="75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="133" t="s">
+    <row r="21" spans="1:8" ht="72" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A21" s="140" t="s">
         <v>836</v>
       </c>
-      <c r="B21" s="127" t="s">
+      <c r="B21" s="143" t="s">
         <v>837</v>
       </c>
-      <c r="C21" s="127" t="s">
+      <c r="C21" s="143" t="s">
         <v>838</v>
       </c>
-      <c r="D21" s="127" t="s">
+      <c r="D21" s="143" t="s">
         <v>839</v>
       </c>
-      <c r="E21" s="127" t="s">
+      <c r="E21" s="192" t="s">
         <v>820</v>
       </c>
-      <c r="F21" s="127" t="s">
+      <c r="F21" s="143" t="s">
         <v>840</v>
       </c>
-      <c r="G21" s="127" t="s">
+      <c r="G21" s="160" t="s">
         <v>834</v>
       </c>
-      <c r="H21" s="127" t="s">
+      <c r="H21" s="155" t="s">
         <v>841</v>
       </c>
     </row>
-    <row r="22" spans="1:8" ht="75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="133" t="s">
+    <row r="22" spans="1:8" ht="72" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A22" s="139" t="s">
         <v>842</v>
       </c>
-      <c r="B22" s="127" t="s">
+      <c r="B22" s="142" t="s">
         <v>843</v>
       </c>
-      <c r="C22" s="127" t="s">
+      <c r="C22" s="142" t="s">
         <v>844</v>
       </c>
-      <c r="D22" s="127" t="s">
+      <c r="D22" s="142" t="s">
         <v>845</v>
       </c>
-      <c r="E22" s="127" t="s">
+      <c r="E22" s="191" t="s">
         <v>820</v>
       </c>
-      <c r="F22" s="127" t="s">
+      <c r="F22" s="142" t="s">
         <v>846</v>
       </c>
-      <c r="G22" s="127" t="s">
+      <c r="G22" s="159" t="s">
         <v>834</v>
       </c>
-      <c r="H22" s="127" t="s">
+      <c r="H22" s="155" t="s">
         <v>847</v>
       </c>
     </row>
-    <row r="23" spans="1:8" ht="75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="133" t="s">
+    <row r="23" spans="1:8" ht="72" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="140" t="s">
         <v>848</v>
       </c>
-      <c r="B23" s="127" t="s">
+      <c r="B23" s="143" t="s">
         <v>849</v>
       </c>
-      <c r="C23" s="127" t="s">
+      <c r="C23" s="143" t="s">
         <v>850</v>
       </c>
-      <c r="D23" s="127" t="s">
+      <c r="D23" s="143" t="s">
         <v>851</v>
       </c>
-      <c r="E23" s="127" t="s">
+      <c r="E23" s="192" t="s">
         <v>852</v>
       </c>
-      <c r="F23" s="127" t="s">
+      <c r="F23" s="143" t="s">
         <v>853</v>
       </c>
-      <c r="G23" s="127" t="s">
+      <c r="G23" s="158" t="s">
         <v>814</v>
       </c>
-      <c r="H23" s="127" t="s">
+      <c r="H23" s="156" t="s">
         <v>854</v>
       </c>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A24" s="127"/>
-      <c r="B24" s="127"/>
-      <c r="C24" s="127"/>
-      <c r="D24" s="127"/>
-      <c r="E24" s="127"/>
-      <c r="F24" s="127"/>
-      <c r="G24" s="127"/>
-      <c r="H24" s="127"/>
-    </row>
-    <row r="25" spans="1:8" ht="22" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:8" ht="8" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A24" s="151"/>
+      <c r="B24" s="151"/>
+      <c r="C24" s="151"/>
+      <c r="D24" s="151"/>
+      <c r="E24" s="151"/>
+      <c r="F24" s="151"/>
+      <c r="G24" s="151"/>
+      <c r="H24" s="150"/>
+    </row>
+    <row r="25" spans="1:8" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A25" s="130" t="s">
         <v>855</v>
       </c>
-      <c r="B25" s="131"/>
-      <c r="C25" s="131"/>
-      <c r="D25" s="131"/>
-      <c r="E25" s="131"/>
-      <c r="F25" s="131"/>
-      <c r="G25" s="131"/>
-      <c r="H25" s="131"/>
-    </row>
-    <row r="26" spans="1:8" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="132" t="s">
+      <c r="B25" s="130"/>
+      <c r="C25" s="130"/>
+      <c r="D25" s="130"/>
+      <c r="E25" s="130"/>
+      <c r="F25" s="130"/>
+      <c r="G25" s="130"/>
+      <c r="H25" s="130"/>
+    </row>
+    <row r="26" spans="1:8" ht="28" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="188" t="s">
         <v>747</v>
       </c>
-      <c r="B26" s="132" t="s">
+      <c r="B26" s="180" t="s">
         <v>856</v>
       </c>
-      <c r="C26" s="132" t="s">
+      <c r="C26" s="180" t="s">
         <v>749</v>
       </c>
-      <c r="D26" s="132" t="s">
+      <c r="D26" s="180" t="s">
         <v>805</v>
       </c>
-      <c r="E26" s="132" t="s">
+      <c r="E26" s="180" t="s">
         <v>857</v>
       </c>
-      <c r="F26" s="132" t="s">
+      <c r="F26" s="180" t="s">
         <v>858</v>
       </c>
-      <c r="G26" s="135"/>
-      <c r="H26" s="132" t="s">
+      <c r="G26" s="179"/>
+      <c r="H26" s="153" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="27" spans="1:8" ht="55" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="133" t="s">
+    <row r="27" spans="1:8" ht="58" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A27" s="141" t="s">
         <v>859</v>
       </c>
-      <c r="B27" s="127" t="s">
+      <c r="B27" s="178" t="s">
         <v>860</v>
       </c>
-      <c r="C27" s="127" t="s">
+      <c r="C27" s="178" t="s">
         <v>861</v>
       </c>
-      <c r="D27" s="127" t="s">
+      <c r="D27" s="178" t="s">
         <v>862</v>
       </c>
-      <c r="E27" s="127" t="s">
+      <c r="E27" s="193" t="s">
         <v>863</v>
       </c>
-      <c r="F27" s="127" t="s">
+      <c r="F27" s="178" t="s">
         <v>864</v>
       </c>
-      <c r="G27" s="127"/>
-      <c r="H27" s="127" t="s">
+      <c r="G27" s="178"/>
+      <c r="H27" s="154" t="s">
         <v>865</v>
       </c>
     </row>
-    <row r="28" spans="1:8" ht="55" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A28" s="133" t="s">
+    <row r="28" spans="1:8" ht="58" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A28" s="139" t="s">
         <v>866</v>
       </c>
-      <c r="B28" s="127" t="s">
+      <c r="B28" s="142" t="s">
         <v>867</v>
       </c>
-      <c r="C28" s="127" t="s">
+      <c r="C28" s="142" t="s">
         <v>868</v>
       </c>
-      <c r="D28" s="127" t="s">
+      <c r="D28" s="142" t="s">
         <v>869</v>
       </c>
-      <c r="E28" s="127" t="s">
+      <c r="E28" s="161" t="s">
         <v>863</v>
       </c>
-      <c r="F28" s="127" t="s">
+      <c r="F28" s="142" t="s">
         <v>870</v>
       </c>
-      <c r="G28" s="127"/>
-      <c r="H28" s="127" t="s">
+      <c r="G28" s="142"/>
+      <c r="H28" s="155" t="s">
         <v>871</v>
       </c>
     </row>
-    <row r="29" spans="1:8" ht="55" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A29" s="133" t="s">
+    <row r="29" spans="1:8" ht="58" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A29" s="140" t="s">
         <v>872</v>
       </c>
-      <c r="B29" s="127" t="s">
+      <c r="B29" s="143" t="s">
         <v>873</v>
       </c>
-      <c r="C29" s="127" t="s">
+      <c r="C29" s="143" t="s">
         <v>874</v>
       </c>
-      <c r="D29" s="127" t="s">
+      <c r="D29" s="143" t="s">
         <v>875</v>
       </c>
-      <c r="E29" s="127" t="s">
+      <c r="E29" s="163" t="s">
         <v>863</v>
       </c>
-      <c r="F29" s="127" t="s">
+      <c r="F29" s="143" t="s">
         <v>876</v>
       </c>
-      <c r="G29" s="127"/>
-      <c r="H29" s="127" t="s">
+      <c r="G29" s="143"/>
+      <c r="H29" s="155" t="s">
         <v>877</v>
       </c>
     </row>
-    <row r="30" spans="1:8" ht="55" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A30" s="133" t="s">
+    <row r="30" spans="1:8" ht="58" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A30" s="139" t="s">
         <v>878</v>
       </c>
-      <c r="B30" s="127" t="s">
+      <c r="B30" s="142" t="s">
         <v>879</v>
       </c>
-      <c r="C30" s="127" t="s">
+      <c r="C30" s="142" t="s">
         <v>880</v>
       </c>
-      <c r="D30" s="127" t="s">
+      <c r="D30" s="142" t="s">
         <v>881</v>
       </c>
-      <c r="E30" s="127" t="s">
+      <c r="E30" s="161" t="s">
         <v>882</v>
       </c>
-      <c r="F30" s="127" t="s">
+      <c r="F30" s="142" t="s">
         <v>883</v>
       </c>
-      <c r="G30" s="127"/>
-      <c r="H30" s="127" t="s">
+      <c r="G30" s="142"/>
+      <c r="H30" s="155" t="s">
         <v>884</v>
       </c>
     </row>
-    <row r="31" spans="1:8" ht="55" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A31" s="133" t="s">
+    <row r="31" spans="1:8" ht="58" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A31" s="140" t="s">
         <v>885</v>
       </c>
-      <c r="B31" s="127" t="s">
+      <c r="B31" s="143" t="s">
         <v>886</v>
       </c>
-      <c r="C31" s="127" t="s">
+      <c r="C31" s="143" t="s">
         <v>887</v>
       </c>
-      <c r="D31" s="127" t="s">
+      <c r="D31" s="143" t="s">
         <v>888</v>
       </c>
-      <c r="E31" s="127" t="s">
+      <c r="E31" s="163" t="s">
         <v>36</v>
       </c>
-      <c r="F31" s="127" t="s">
+      <c r="F31" s="143" t="s">
         <v>889</v>
       </c>
-      <c r="G31" s="127"/>
-      <c r="H31" s="127" t="s">
+      <c r="G31" s="143"/>
+      <c r="H31" s="155" t="s">
         <v>890</v>
       </c>
     </row>
-    <row r="32" spans="1:8" ht="55" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A32" s="133" t="s">
+    <row r="32" spans="1:8" ht="58" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="139" t="s">
         <v>891</v>
       </c>
-      <c r="B32" s="127" t="s">
+      <c r="B32" s="142" t="s">
         <v>892</v>
       </c>
-      <c r="C32" s="127" t="s">
+      <c r="C32" s="142" t="s">
         <v>893</v>
       </c>
-      <c r="D32" s="127" t="s">
+      <c r="D32" s="142" t="s">
         <v>894</v>
       </c>
-      <c r="E32" s="127" t="s">
+      <c r="E32" s="161" t="s">
         <v>36</v>
       </c>
-      <c r="F32" s="127" t="s">
+      <c r="F32" s="142" t="s">
         <v>895</v>
       </c>
-      <c r="G32" s="127"/>
-      <c r="H32" s="127" t="s">
+      <c r="G32" s="142"/>
+      <c r="H32" s="156" t="s">
         <v>896</v>
       </c>
     </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A33" s="127"/>
-      <c r="B33" s="127"/>
-      <c r="C33" s="127"/>
-      <c r="D33" s="127"/>
-      <c r="E33" s="127"/>
-      <c r="F33" s="127"/>
-      <c r="G33" s="127"/>
-      <c r="H33" s="127"/>
-    </row>
-    <row r="34" spans="1:8" ht="22" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:8" ht="8" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A33" s="151"/>
+      <c r="B33" s="151"/>
+      <c r="C33" s="151"/>
+      <c r="D33" s="151"/>
+      <c r="E33" s="151"/>
+      <c r="F33" s="151"/>
+      <c r="G33" s="151"/>
+      <c r="H33" s="150"/>
+    </row>
+    <row r="34" spans="1:8" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A34" s="130" t="s">
         <v>897</v>
       </c>
-      <c r="B34" s="131"/>
-      <c r="C34" s="131"/>
-      <c r="D34" s="131"/>
-      <c r="E34" s="131"/>
-      <c r="F34" s="131"/>
-      <c r="G34" s="131"/>
-      <c r="H34" s="131"/>
-    </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A35" s="127"/>
-      <c r="B35" s="127"/>
-      <c r="C35" s="127"/>
-      <c r="D35" s="127"/>
-      <c r="E35" s="127"/>
-      <c r="F35" s="127"/>
-      <c r="G35" s="127"/>
-      <c r="H35" s="127"/>
-    </row>
-    <row r="36" spans="1:8" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A36" s="132" t="s">
+      <c r="B34" s="130"/>
+      <c r="C34" s="130"/>
+      <c r="D34" s="130"/>
+      <c r="E34" s="130"/>
+      <c r="F34" s="130"/>
+      <c r="G34" s="130"/>
+      <c r="H34" s="130"/>
+    </row>
+    <row r="35" spans="1:8" ht="8" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A35" s="152"/>
+      <c r="B35" s="152"/>
+      <c r="C35" s="152"/>
+      <c r="D35" s="152"/>
+      <c r="E35" s="152"/>
+      <c r="F35" s="152"/>
+      <c r="G35" s="152"/>
+      <c r="H35" s="152"/>
+    </row>
+    <row r="36" spans="1:8" ht="28" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A36" s="189" t="s">
         <v>898</v>
       </c>
-      <c r="B36" s="132" t="s">
+      <c r="B36" s="185" t="s">
         <v>62</v>
       </c>
-      <c r="C36" s="132" t="s">
+      <c r="C36" s="183" t="s">
         <v>899</v>
       </c>
-      <c r="D36" s="132" t="s">
+      <c r="D36" s="131" t="s">
         <v>61</v>
       </c>
-      <c r="E36" s="127"/>
-      <c r="F36" s="127"/>
-      <c r="G36" s="127"/>
-      <c r="H36" s="127"/>
-    </row>
-    <row r="37" spans="1:8" ht="55" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A37" s="136" t="s">
+      <c r="E36" s="150"/>
+      <c r="F36" s="150"/>
+      <c r="G36" s="150"/>
+      <c r="H36" s="150"/>
+    </row>
+    <row r="37" spans="1:8" ht="42" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A37" s="146" t="s">
         <v>900</v>
       </c>
-      <c r="B37" s="127" t="s">
+      <c r="B37" s="178" t="s">
         <v>901</v>
       </c>
-      <c r="C37" s="137" t="s">
+      <c r="C37" s="186" t="s">
         <v>902</v>
       </c>
-      <c r="D37" s="127" t="s">
+      <c r="D37" s="132" t="s">
         <v>814</v>
       </c>
-      <c r="E37" s="127"/>
-      <c r="F37" s="127"/>
-      <c r="G37" s="127"/>
-      <c r="H37" s="127"/>
-    </row>
-    <row r="38" spans="1:8" ht="55" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A38" s="136" t="s">
+      <c r="E37" s="150"/>
+      <c r="F37" s="150"/>
+      <c r="G37" s="150"/>
+      <c r="H37" s="150"/>
+    </row>
+    <row r="38" spans="1:8" ht="42" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A38" s="144" t="s">
         <v>903</v>
       </c>
-      <c r="B38" s="127" t="s">
+      <c r="B38" s="142" t="s">
         <v>904</v>
       </c>
-      <c r="C38" s="137" t="s">
+      <c r="C38" s="167" t="s">
         <v>905</v>
       </c>
-      <c r="D38" s="127" t="s">
+      <c r="D38" s="133" t="s">
         <v>814</v>
       </c>
-      <c r="E38" s="127"/>
-      <c r="F38" s="127"/>
-      <c r="G38" s="127"/>
-      <c r="H38" s="127"/>
-    </row>
-    <row r="39" spans="1:8" ht="55" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A39" s="136" t="s">
+      <c r="E38" s="150"/>
+      <c r="F38" s="150"/>
+      <c r="G38" s="150"/>
+      <c r="H38" s="150"/>
+    </row>
+    <row r="39" spans="1:8" ht="42" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A39" s="145" t="s">
         <v>906</v>
       </c>
-      <c r="B39" s="127" t="s">
+      <c r="B39" s="143" t="s">
         <v>907</v>
       </c>
-      <c r="C39" s="137" t="s">
+      <c r="C39" s="168" t="s">
         <v>908</v>
       </c>
-      <c r="D39" s="127" t="s">
+      <c r="D39" s="134" t="s">
         <v>834</v>
       </c>
-      <c r="E39" s="127"/>
-      <c r="F39" s="127"/>
-      <c r="G39" s="127"/>
-      <c r="H39" s="127"/>
-    </row>
-    <row r="40" spans="1:8" ht="55" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A40" s="136" t="s">
+      <c r="E39" s="150"/>
+      <c r="F39" s="150"/>
+      <c r="G39" s="150"/>
+      <c r="H39" s="150"/>
+    </row>
+    <row r="40" spans="1:8" ht="42" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A40" s="144" t="s">
         <v>909</v>
       </c>
-      <c r="B40" s="127" t="s">
+      <c r="B40" s="142" t="s">
         <v>910</v>
       </c>
-      <c r="C40" s="138" t="s">
+      <c r="C40" s="170" t="s">
         <v>911</v>
       </c>
-      <c r="D40" s="127" t="s">
+      <c r="D40" s="135" t="s">
         <v>912</v>
       </c>
-      <c r="E40" s="127"/>
-      <c r="F40" s="127"/>
-      <c r="G40" s="127"/>
-      <c r="H40" s="127"/>
-    </row>
-    <row r="41" spans="1:8" ht="55" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A41" s="136" t="s">
+      <c r="E40" s="150"/>
+      <c r="F40" s="150"/>
+      <c r="G40" s="150"/>
+      <c r="H40" s="150"/>
+    </row>
+    <row r="41" spans="1:8" ht="42" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A41" s="145" t="s">
         <v>913</v>
       </c>
-      <c r="B41" s="127" t="s">
+      <c r="B41" s="143" t="s">
         <v>914</v>
       </c>
-      <c r="C41" s="137" t="s">
+      <c r="C41" s="168" t="s">
         <v>915</v>
       </c>
-      <c r="D41" s="127" t="s">
+      <c r="D41" s="134" t="s">
         <v>834</v>
       </c>
-      <c r="E41" s="127"/>
-      <c r="F41" s="127"/>
-      <c r="G41" s="127"/>
-      <c r="H41" s="127"/>
-    </row>
-    <row r="42" spans="1:8" ht="55" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A42" s="136" t="s">
+      <c r="E41" s="150"/>
+      <c r="F41" s="150"/>
+      <c r="G41" s="150"/>
+      <c r="H41" s="150"/>
+    </row>
+    <row r="42" spans="1:8" ht="42" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A42" s="144" t="s">
         <v>916</v>
       </c>
-      <c r="B42" s="127" t="s">
+      <c r="B42" s="142" t="s">
         <v>917</v>
       </c>
-      <c r="C42" s="139" t="s">
+      <c r="C42" s="169" t="s">
         <v>918</v>
       </c>
-      <c r="D42" s="127" t="s">
+      <c r="D42" s="133" t="s">
         <v>814</v>
       </c>
-      <c r="E42" s="127"/>
-      <c r="F42" s="127"/>
-      <c r="G42" s="127"/>
-      <c r="H42" s="127"/>
-    </row>
-    <row r="43" spans="1:8" ht="55" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A43" s="136" t="s">
+      <c r="E42" s="150"/>
+      <c r="F42" s="150"/>
+      <c r="G42" s="150"/>
+      <c r="H42" s="150"/>
+    </row>
+    <row r="43" spans="1:8" ht="42" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A43" s="145" t="s">
         <v>919</v>
       </c>
-      <c r="B43" s="127" t="s">
+      <c r="B43" s="143" t="s">
         <v>920</v>
       </c>
-      <c r="C43" s="137" t="s">
+      <c r="C43" s="168" t="s">
         <v>921</v>
       </c>
-      <c r="D43" s="127" t="s">
+      <c r="D43" s="137" t="s">
         <v>814</v>
       </c>
-      <c r="E43" s="127"/>
-      <c r="F43" s="127"/>
-      <c r="G43" s="127"/>
-      <c r="H43" s="127"/>
-    </row>
-    <row r="44" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A44" s="127"/>
-      <c r="B44" s="127"/>
-      <c r="C44" s="127"/>
-      <c r="D44" s="127"/>
-      <c r="E44" s="127"/>
-      <c r="F44" s="127"/>
-      <c r="G44" s="127"/>
-      <c r="H44" s="127"/>
-    </row>
-    <row r="45" spans="1:8" ht="22" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="E43" s="150"/>
+      <c r="F43" s="150"/>
+      <c r="G43" s="150"/>
+      <c r="H43" s="150"/>
+    </row>
+    <row r="44" spans="1:8" ht="8" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A44" s="150"/>
+      <c r="B44" s="150"/>
+      <c r="C44" s="150"/>
+      <c r="D44" s="150"/>
+      <c r="E44" s="150"/>
+      <c r="F44" s="150"/>
+      <c r="G44" s="150"/>
+      <c r="H44" s="150"/>
+    </row>
+    <row r="45" spans="1:8" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A45" s="130" t="s">
         <v>922</v>
       </c>
-      <c r="B45" s="131"/>
-      <c r="C45" s="131"/>
-      <c r="D45" s="131"/>
-      <c r="E45" s="131"/>
-      <c r="F45" s="131"/>
-      <c r="G45" s="131"/>
-      <c r="H45" s="131"/>
-    </row>
-    <row r="46" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A46" s="127"/>
-      <c r="B46" s="127"/>
-      <c r="C46" s="127"/>
-      <c r="D46" s="127"/>
-      <c r="E46" s="127"/>
-      <c r="F46" s="127"/>
-      <c r="G46" s="127"/>
-      <c r="H46" s="127"/>
-    </row>
-    <row r="47" spans="1:8" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A47" s="132" t="s">
+      <c r="B45" s="130"/>
+      <c r="C45" s="130"/>
+      <c r="D45" s="130"/>
+      <c r="E45" s="130"/>
+      <c r="F45" s="130"/>
+      <c r="G45" s="130"/>
+      <c r="H45" s="130"/>
+    </row>
+    <row r="46" spans="1:8" ht="8" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A46" s="152"/>
+      <c r="B46" s="152"/>
+      <c r="C46" s="152"/>
+      <c r="D46" s="152"/>
+      <c r="E46" s="152"/>
+      <c r="F46" s="152"/>
+      <c r="G46" s="152"/>
+      <c r="H46" s="152"/>
+    </row>
+    <row r="47" spans="1:8" ht="28" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A47" s="189" t="s">
         <v>31</v>
       </c>
-      <c r="B47" s="132" t="s">
+      <c r="B47" s="185" t="s">
         <v>923</v>
       </c>
-      <c r="C47" s="132" t="s">
+      <c r="C47" s="183" t="s">
         <v>924</v>
       </c>
-      <c r="D47" s="132" t="s">
+      <c r="D47" s="131" t="s">
         <v>61</v>
       </c>
-      <c r="E47" s="127"/>
-      <c r="F47" s="127"/>
-      <c r="G47" s="127"/>
-      <c r="H47" s="127"/>
+      <c r="E47" s="150"/>
+      <c r="F47" s="150"/>
+      <c r="G47" s="150"/>
+      <c r="H47" s="150"/>
     </row>
     <row r="48" spans="1:8" ht="65" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A48" s="133" t="s">
+      <c r="A48" s="146" t="s">
         <v>925</v>
       </c>
-      <c r="B48" s="136" t="s">
+      <c r="B48" s="184" t="s">
         <v>926</v>
       </c>
-      <c r="C48" s="136" t="s">
+      <c r="C48" s="187" t="s">
         <v>927</v>
       </c>
-      <c r="D48" s="140" t="s">
+      <c r="D48" s="136" t="s">
         <v>834</v>
       </c>
-      <c r="E48" s="127"/>
-      <c r="F48" s="127"/>
-      <c r="G48" s="127"/>
-      <c r="H48" s="127"/>
+      <c r="E48" s="150"/>
+      <c r="F48" s="150"/>
+      <c r="G48" s="150"/>
+      <c r="H48" s="150"/>
     </row>
     <row r="49" spans="1:8" ht="65" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A49" s="133" t="s">
+      <c r="A49" s="144" t="s">
         <v>928</v>
       </c>
-      <c r="B49" s="136" t="s">
+      <c r="B49" s="171" t="s">
         <v>929</v>
       </c>
-      <c r="C49" s="136" t="s">
+      <c r="C49" s="175" t="s">
         <v>930</v>
       </c>
-      <c r="D49" s="140" t="s">
+      <c r="D49" s="135" t="s">
         <v>912</v>
       </c>
-      <c r="E49" s="127"/>
-      <c r="F49" s="127"/>
-      <c r="G49" s="127"/>
-      <c r="H49" s="127"/>
+      <c r="E49" s="150"/>
+      <c r="F49" s="150"/>
+      <c r="G49" s="150"/>
+      <c r="H49" s="150"/>
     </row>
     <row r="50" spans="1:8" ht="65" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A50" s="133" t="s">
+      <c r="A50" s="145" t="s">
         <v>931</v>
       </c>
-      <c r="B50" s="136" t="s">
+      <c r="B50" s="172" t="s">
         <v>932</v>
       </c>
-      <c r="C50" s="136" t="s">
+      <c r="C50" s="176" t="s">
         <v>933</v>
       </c>
-      <c r="D50" s="140" t="s">
+      <c r="D50" s="137" t="s">
         <v>814</v>
       </c>
-      <c r="E50" s="127"/>
-      <c r="F50" s="127"/>
-      <c r="G50" s="127"/>
-      <c r="H50" s="127"/>
+      <c r="E50" s="150"/>
+      <c r="F50" s="150"/>
+      <c r="G50" s="150"/>
+      <c r="H50" s="150"/>
     </row>
     <row r="51" spans="1:8" ht="65" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A51" s="133" t="s">
+      <c r="A51" s="144" t="s">
         <v>934</v>
       </c>
-      <c r="B51" s="136" t="s">
+      <c r="B51" s="171" t="s">
         <v>935</v>
       </c>
-      <c r="C51" s="136" t="s">
+      <c r="C51" s="175" t="s">
         <v>936</v>
       </c>
-      <c r="D51" s="140" t="s">
+      <c r="D51" s="133" t="s">
         <v>814</v>
       </c>
-      <c r="E51" s="127"/>
-      <c r="F51" s="127"/>
-      <c r="G51" s="127"/>
-      <c r="H51" s="127"/>
+      <c r="E51" s="150"/>
+      <c r="F51" s="150"/>
+      <c r="G51" s="150"/>
+      <c r="H51" s="150"/>
     </row>
     <row r="52" spans="1:8" ht="65" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A52" s="133" t="s">
+      <c r="A52" s="145" t="s">
         <v>937</v>
       </c>
-      <c r="B52" s="136" t="s">
+      <c r="B52" s="172" t="s">
         <v>938</v>
       </c>
-      <c r="C52" s="136" t="s">
+      <c r="C52" s="176" t="s">
         <v>939</v>
       </c>
-      <c r="D52" s="140" t="s">
+      <c r="D52" s="137" t="s">
         <v>814</v>
       </c>
-      <c r="E52" s="127"/>
-      <c r="F52" s="127"/>
-      <c r="G52" s="127"/>
-      <c r="H52" s="127"/>
+      <c r="E52" s="150"/>
+      <c r="F52" s="150"/>
+      <c r="G52" s="150"/>
+      <c r="H52" s="150"/>
     </row>
     <row r="53" spans="1:8" ht="65" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A53" s="133" t="s">
+      <c r="A53" s="144" t="s">
         <v>940</v>
       </c>
-      <c r="B53" s="136" t="s">
+      <c r="B53" s="171" t="s">
         <v>941</v>
       </c>
-      <c r="C53" s="136" t="s">
+      <c r="C53" s="175" t="s">
         <v>942</v>
       </c>
-      <c r="D53" s="140" t="s">
+      <c r="D53" s="133" t="s">
         <v>814</v>
       </c>
-      <c r="E53" s="127"/>
-      <c r="F53" s="127"/>
-      <c r="G53" s="127"/>
-      <c r="H53" s="127"/>
-    </row>
-    <row r="54" spans="1:8" ht="65" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A54" s="133" t="s">
+      <c r="E53" s="150"/>
+      <c r="F53" s="150"/>
+      <c r="G53" s="150"/>
+      <c r="H53" s="150"/>
+    </row>
+    <row r="54" spans="1:8" ht="65" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A54" s="149" t="s">
         <v>943</v>
       </c>
-      <c r="B54" s="136" t="s">
+      <c r="B54" s="173" t="s">
         <v>944</v>
       </c>
-      <c r="C54" s="136" t="s">
+      <c r="C54" s="177" t="s">
         <v>945</v>
       </c>
-      <c r="D54" s="140" t="s">
+      <c r="D54" s="138" t="s">
         <v>912</v>
       </c>
-      <c r="E54" s="127"/>
-      <c r="F54" s="127"/>
-      <c r="G54" s="127"/>
-      <c r="H54" s="127"/>
-    </row>
-    <row r="55" spans="1:8" ht="85" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A55" s="141" t="s">
+      <c r="E54" s="150"/>
+      <c r="F54" s="150"/>
+      <c r="G54" s="150"/>
+      <c r="H54" s="150"/>
+    </row>
+    <row r="55" spans="1:8" ht="85" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A55" s="148" t="s">
         <v>60</v>
       </c>
-      <c r="B55" s="132" t="s">
+      <c r="B55" s="174" t="s">
         <v>946</v>
       </c>
-      <c r="C55" s="132" t="s">
+      <c r="C55" s="174" t="s">
         <v>947</v>
       </c>
-      <c r="D55" s="142" t="s">
+      <c r="D55" s="147" t="s">
         <v>834</v>
       </c>
-      <c r="E55" s="127"/>
-      <c r="F55" s="127"/>
-      <c r="G55" s="127"/>
-      <c r="H55" s="127"/>
+      <c r="E55" s="150"/>
+      <c r="F55" s="150"/>
+      <c r="G55" s="150"/>
+      <c r="H55" s="150"/>
     </row>
   </sheetData>
+  <mergeCells count="8">
+    <mergeCell ref="A34:H34"/>
+    <mergeCell ref="A45:H45"/>
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A3:H3"/>
+    <mergeCell ref="A5:H5"/>
+    <mergeCell ref="A15:H15"/>
+    <mergeCell ref="A25:H25"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <legacyDrawing r:id="rId1"/>
 </worksheet>
@@ -13424,7 +14115,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F24F8A94-CAFB-ED4A-8BD7-5C46C6CC39CB}">
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:F10"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="8.33203125" customWidth="1"/>
@@ -13615,6 +14306,26 @@
         <v>951</v>
       </c>
     </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10" s="46">
+        <v>46085</v>
+      </c>
+      <c r="C10" t="s">
+        <v>952</v>
+      </c>
+      <c r="D10" t="s">
+        <v>953</v>
+      </c>
+      <c r="E10" t="s">
+        <v>954</v>
+      </c>
+      <c r="F10" t="s">
+        <v>955</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>